<commit_message>
docs(j3): ajout veille sécurité, scénarios audit/test, MAJ sprint backlog + pages légales RGPD
</commit_message>
<xml_diff>
--- a/docs/perturbations/j3/sprint-backlog.xlsx
+++ b/docs/perturbations/j3/sprint-backlog.xlsx
@@ -1,17 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Garde" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identification" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Burndown Sprint 1" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auto-évaluation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Garde" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Identification" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sprint 1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Burndown Sprint 1" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sprint 5" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Burndown Sprint 5" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Auto-évaluation" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -687,7 +689,7 @@
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Décomposition technique du Sprint 1 d'EduTutor IA (lundi 14h-18h)</t>
+          <t>Décomposition technique des sprints d'EduTutor IA — Sprint 1 (cadrage) + Sprint 5 (perturbation J3)</t>
         </is>
       </c>
     </row>
@@ -770,7 +772,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Cadrage</t>
+          <t>Sprint 5 (perturbation J3)</t>
         </is>
       </c>
     </row>
@@ -782,7 +784,7 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>v2.0</t>
+          <t>v3.0</t>
         </is>
       </c>
     </row>
@@ -794,7 +796,7 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>30/06/2026  17h45</t>
+          <t>01/07/2026  17h45</t>
         </is>
       </c>
     </row>
@@ -1708,6 +1710,979 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>SPRINT BACKLOG : SPRINT 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Mercredi 01/07/2026 · MVP + perturbation J3 (OWASP LLM-01 Prompt Injection + SAR RGPD) · 28 h-pers</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>📋 MÉTADONNÉES DU SPRINT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Numéro de sprint</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Mercredi 01/07/2026 (livraison MVP 17h45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Équipe (n personnes)</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>7 personnes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Capacité totale</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>7 × 4 h = 28 h-pers (slice J3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Vélocité cible (SP)</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>9 SP J3 MUST — US-24 (2), US-25 (3), US-26 (3), US-27 (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Objectif sprint</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Intégrer la sécurité LLM (4 couches OWASP LLM-01) et l'export RGPD (SAR Art. 15/20) à la livraison MVP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Scrum Master</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>[ à désigner en équipe ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>[ PO externe, à renseigner ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>💡 OBJECTIF</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Décomposer chaque story tirée du Product Backlog en tâches techniques fines (1-3h), avec assignation et estimation. Mis à jour en daily.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>📐 FORMAT</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>3 à 5 tâches par user story. Estimation en heures (pas SP, trop grossier pour 1 sprint court). Restant mis à jour à chaque daily.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>✅ BON</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>« T-25.1 Écrire 5 tests adversariaux pytest (clair, base64, multilingue, blanc/blanc, Unicode) — Amine — 3 h »</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>❌ À ÉVITER</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>« Faire l'inscription » (pas de tâche atomique, ni assigné, ni estimable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>ID tâche</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Tâche technique</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Assigné</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Estim. (h)</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Restant (h)</t>
+        </is>
+      </c>
+      <c r="G19" s="18" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>US-24</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>T-24.1</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>Rédiger la section « SÉCURITÉ (OWASP LLM-01) » dans SYSTEM_PROMPT</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>Alexandre</t>
+        </is>
+      </c>
+      <c r="E20" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>US-24</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>T-24.2</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>Refactor build_user_prompt()/build_full_prompt() (séparation system/user)</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>Valentin</t>
+        </is>
+      </c>
+      <c r="E21" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>US-24</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>T-24.3</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>Adapter les clients LLM (2 messages role-based vs prompt completion)</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>Bastien</t>
+        </is>
+      </c>
+      <c r="E22" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>US-25</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>T-25.1</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>Écrire les 5 tests adversariaux pytest (clair, base64, multilingue, blanc/blanc, Unicode)</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>Amine</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>US-25</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>T-25.2</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="inlineStr">
+        <is>
+          <t>Validation stricte parse_and_validate_quiz() (10 Q × 4 options × correct_index)</t>
+        </is>
+      </c>
+      <c r="D24" s="23" t="inlineStr">
+        <is>
+          <t>Erwann</t>
+        </is>
+      </c>
+      <c r="E24" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>US-25</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>T-25.3</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>generate_quiz_with_retry() (plafond 2 tentatives puis 502)</t>
+        </is>
+      </c>
+      <c r="D25" s="23" t="inlineStr">
+        <is>
+          <t>Erwann</t>
+        </is>
+      </c>
+      <c r="E25" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>US-25</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>T-25.4</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="inlineStr">
+        <is>
+          <t>Step CI « Adversarial security tests » dans .github/workflows/ci.yml</t>
+        </is>
+      </c>
+      <c r="D26" s="23" t="inlineStr">
+        <is>
+          <t>Evan</t>
+        </is>
+      </c>
+      <c r="E26" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>US-26</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>T-26.1</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>Endpoint GET /api/accounts/me/export/ (JSON + Content-Disposition attachment)</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>Aya</t>
+        </is>
+      </c>
+      <c r="E27" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>US-26</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>T-26.2</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>Audit trail SAR (log structuré IP + email + id + timestamp)</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>Evan</t>
+        </is>
+      </c>
+      <c r="E28" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>US-26</t>
+        </is>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>T-26.3</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>Tests pytest export RGPD + vérification de l'audit trail</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>Alexandre</t>
+        </is>
+      </c>
+      <c r="E29" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>US-27</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>T-27.1</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
+          <t>Rédiger politique-retention.md (mapping Art. 15/16/17/18/20 + durées)</t>
+        </is>
+      </c>
+      <c r="D30" s="23" t="inlineStr">
+        <is>
+          <t>Valentin</t>
+        </is>
+      </c>
+      <c r="E30" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>US-27</t>
+        </is>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>T-27.2</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="inlineStr">
+        <is>
+          <t>Relecture PO + note de décision MoSCoW J3</t>
+        </is>
+      </c>
+      <c r="D31" s="23" t="inlineStr">
+        <is>
+          <t>Bastien</t>
+        </is>
+      </c>
+      <c r="E31" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="25" t="inlineStr"/>
+      <c r="B32" s="25" t="inlineStr"/>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>[ Sprint 5 livré — 12 tâches, toutes Done au 01/07 17h45 ]</t>
+        </is>
+      </c>
+      <c r="D32" s="26" t="inlineStr"/>
+      <c r="E32" s="27" t="inlineStr"/>
+      <c r="F32" s="27" t="inlineStr"/>
+      <c r="G32" s="26" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="28" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B33" s="29" t="n"/>
+      <c r="C33" s="30" t="inlineStr">
+        <is>
+          <t>18 h estimées · capacité 28 h-pers · marge 10 h (livraison MVP menée en parallèle)</t>
+        </is>
+      </c>
+      <c r="D33" s="29" t="n"/>
+      <c r="E33" s="28" t="n">
+        <v>18</v>
+      </c>
+      <c r="F33" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="29" t="n"/>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>📌 STATUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="31" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Tâche pas encore commencée</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="32" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Tâche en cours (1 seule par personne idéalement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Tâche bloquée, à remonter en daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Tâche terminée et validée</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>BURNDOWN : SPRINT 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Trajectoire des heures restantes du slice J3 le 01/07/2026 (18 h → 0 h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>💡 BURNDOWN vs BURNUP</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Le BURNDOWN trace les h-pers restantes au cours du sprint (descendant). Burnup = livré cumulé (montant). Pour 1 sprint court, burndown est plus actionnable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>📐 LECTURE</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Idéal : descente linéaire de 18 h (estim.) à 0 h. Réel : à reporter à chaque daily.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Moment du sprint</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Heure restante (idéal)</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Heure restante (réel)</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Δ réel-idéal</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>14h00, Début sprint</t>
+        </is>
+      </c>
+      <c r="B8" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="C8" s="34" t="n">
+        <v>18</v>
+      </c>
+      <c r="D8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>Début sprint, toutes tâches en Todo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>15h00, Daily intermédiaire</t>
+        </is>
+      </c>
+      <c r="B9" s="34" t="n">
+        <v>14</v>
+      </c>
+      <c r="C9" s="34" t="n">
+        <v>13</v>
+      </c>
+      <c r="D9" s="34" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>1/4 du sprint écoulé</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="25" customHeight="1">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>16h00, Mi-sprint</t>
+        </is>
+      </c>
+      <c r="B10" s="34" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="34" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>Mi-sprint, point de vigilance</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>17h00, Avant clôture</t>
+        </is>
+      </c>
+      <c r="B11" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="34" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Dernière heure, finition tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>18h00, Fin sprint / Review</t>
+        </is>
+      </c>
+      <c r="B12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Review + démo PO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>📊 INSÉRER UN GRAPHIQUE</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Sélectionnez les colonnes Moment / Idéal / Réel puis Excel : Insertion &gt; Graphique en courbes. 2 séries (Idéal en pointillés, Réel en plein). L'écart visualise la dérive du sprint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>📈 LECTURE DE LA COURBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Réel ≈ Idéal</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Sprint sous contrôle, vélocité conforme à l'estimation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>Réel &gt; Idéal</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Retard, réfléchir en daily à un re-planning ou retrait d'une tâche non critique</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>Réel &lt; Idéal</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Avance, possibilité de tirer une tâche supplémentaire du Product Backlog</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Courbe plate</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Tâches bloquées, escalader immédiatement avec le Scrum Master</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A2:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>